<commit_message>
Add .gitignore and exclude .env and venv
</commit_message>
<xml_diff>
--- a/binance_trades.xlsx
+++ b/binance_trades.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -679,6 +679,104 @@
       </c>
       <c r="K5" t="n">
         <v>1772260354981</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BTCUSDT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>02-03-2026 02:30:24</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>8</v>
+      </c>
+      <c r="I6" t="n">
+        <v>65333.3</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1772398971672</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ETHUSDT</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>02-03-2026 11:44:59</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>LIMIT</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>111.111</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1968.88</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1772432114670</v>
       </c>
     </row>
   </sheetData>

</xml_diff>